<commit_message>
A "lot" of progress
Fetching works I guess, and uploading works half-way
Maybe we'll do this
</commit_message>
<xml_diff>
--- a/ultetheto_novenyek.xlsx
+++ b/ultetheto_novenyek.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admill\Documents\GitHub\GardenPlanner-March6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F84C009-261C-4AE5-A300-8CD76ED8BAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C54F4D-A518-4BF1-BCEA-97FA8C37EEB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
That's all I'm willing to do for now
At this point I don't care what grades we get, if we'll even present it. If we get another week, optimization and upgrading will be the main focus.
</commit_message>
<xml_diff>
--- a/ultetheto_novenyek.xlsx
+++ b/ultetheto_novenyek.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admill\Documents\GitHub\GardenPlanner-March6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C54F4D-A518-4BF1-BCEA-97FA8C37EEB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A47D21A-24EA-4368-99F7-46E02CC253A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="156" yWindow="228" windowWidth="22884" windowHeight="11340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -220,7 +220,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -230,12 +230,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -267,13 +261,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -636,7 +629,7 @@
       <c r="F2" s="2">
         <v>40</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -662,7 +655,7 @@
       <c r="F3" s="2">
         <v>50</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>49</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -688,7 +681,7 @@
       <c r="F4" s="2">
         <v>20</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>50</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -714,7 +707,7 @@
       <c r="F5" s="2">
         <v>30</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -722,54 +715,54 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>25</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
         <v>75</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="2" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>